<commit_message>
fix timeseries gdp value formatting
</commit_message>
<xml_diff>
--- a/input/config.xlsx
+++ b/input/config.xlsx
@@ -8986,7 +8986,7 @@
         <v>214</v>
       </c>
       <c r="B107" s="3" t="n">
-        <v>36311882</v>
+        <v>36311882000000</v>
       </c>
       <c r="C107" s="5" t="s">
         <v>215</v>
@@ -9019,7 +9019,7 @@
         <v>216</v>
       </c>
       <c r="B108" s="3" t="n">
-        <v>39335929</v>
+        <v>39335929000000</v>
       </c>
       <c r="C108" s="5" t="s">
         <v>215</v>
@@ -9052,7 +9052,7 @@
         <v>217</v>
       </c>
       <c r="B109" s="3" t="n">
-        <v>43553984</v>
+        <v>43553984000000</v>
       </c>
       <c r="C109" s="5" t="s">
         <v>215</v>
@@ -9085,7 +9085,7 @@
         <v>218</v>
       </c>
       <c r="B110" s="3" t="n">
-        <v>47940496</v>
+        <v>47940496000000</v>
       </c>
       <c r="C110" s="5" t="s">
         <v>215</v>
@@ -9118,7 +9118,7 @@
         <v>219</v>
       </c>
       <c r="B111" s="3" t="n">
-        <v>48807766</v>
+        <v>48807766000000</v>
       </c>
       <c r="C111" s="5" t="s">
         <v>215</v>
@@ -9151,7 +9151,7 @@
         <v>220</v>
       </c>
       <c r="B112" s="3" t="n">
-        <v>55560466</v>
+        <v>55560466000000</v>
       </c>
       <c r="C112" s="5" t="s">
         <v>215</v>
@@ -9184,7 +9184,7 @@
         <v>221</v>
       </c>
       <c r="B113" s="3" t="n">
-        <v>65950424</v>
+        <v>65950424000000</v>
       </c>
       <c r="C113" s="5" t="s">
         <v>215</v>
@@ -9217,7 +9217,7 @@
         <v>222</v>
       </c>
       <c r="B114" s="3" t="n">
-        <v>75292668</v>
+        <v>75292668000000</v>
       </c>
       <c r="C114" s="5" t="s">
         <v>215</v>
@@ -9250,7 +9250,7 @@
         <v>223</v>
       </c>
       <c r="B115" s="3" t="n">
-        <v>81447664</v>
+        <v>81447664000000</v>
       </c>
       <c r="C115" s="5" t="s">
         <v>215</v>

</xml_diff>